<commit_message>
Aufgabe 33 (Block 10) ueberarbeitet: Zielbeschreibung, Verstaendnisfragen, vereinfachtes Zaehlen
Zielbeschreibung praezisiert (konkrete, wachsende Arrays statt nur
abstrakter Komplexitaetsbezug), Hilfsfunktion vergleicheZahlen entfernt
und das Mitzaehlen direkt in teileMitZaehler eingebaut, neuer Schritt 1
mit vier Verstaendnisfragen zur main-Funktion vor der Programmausfuehrung.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/02-theoriephase/termin-05/code/vorlage-33-komplexitaetsvergleich.xlsx
+++ b/docs/02-theoriephase/termin-05/code/vorlage-33-komplexitaetsvergleich.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstoecker\AppData\Local\Temp\gt\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CGT\Lehre\GDI\docs\02-theoriephase\termin-05\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A1AE6C-A8FA-45A5-8111-2EC0869E737F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF712119-0253-4E84-A1A6-A7D9C5305DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -219,7 +219,7 @@
     <c:title>
       <c:tx>
         <c:rich>
-          <a:bodyPr/>
+          <a:bodyPr anchor="t" anchorCtr="0"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
@@ -232,11 +232,29 @@
           </a:p>
         </c:rich>
       </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.39932082018306148"/>
+          <c:y val="1.7561443735047134E-2"/>
+        </c:manualLayout>
+      </c:layout>
       <c:overlay val="1"/>
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.6846008031733882E-2"/>
+          <c:y val="0.10274182073453389"/>
+          <c:w val="0.89836159066704302"/>
+          <c:h val="0.80915089497680481"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -570,6 +588,14 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.47573093204411077"/>
+              <c:y val="0.93238106673556043"/>
+            </c:manualLayout>
+          </c:layout>
           <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
@@ -588,13 +614,13 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines/>
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr/>
+              <a:bodyPr anchor="t" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -607,6 +633,14 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="8.0685825279398493E-3"/>
+              <c:y val="0.37624837962962965"/>
+            </c:manualLayout>
+          </c:layout>
           <c:overlay val="1"/>
         </c:title>
         <c:numFmt formatCode="#,##0" sourceLinked="1"/>
@@ -640,10 +674,10 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>157161</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="8640000" cy="4320000"/>
+    <xdr:ext cx="9444038" cy="4339051"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">

</xml_diff>